<commit_message>
Writing data to Csv using pandas
</commit_message>
<xml_diff>
--- a/newData.xlsx
+++ b/newData.xlsx
@@ -9,10 +9,10 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12180" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12180"/>
   </bookViews>
   <sheets>
-    <sheet name="sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>

</xml_diff>